<commit_message>
added new module for SEM
</commit_message>
<xml_diff>
--- a/SEM Automation Scripts/SEM Validation Report/SEM Validation Report 2024-10-28.xlsx
+++ b/SEM Automation Scripts/SEM Validation Report/SEM Validation Report 2024-10-28.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shubham.puri\Genentech\SEM Automation Scripts\SEM Validation Report\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://perficient-my.sharepoint.com/personal/shubham_puri_perficient_com/Documents/Excel VBA Automation/SEM Automation Scripts/SEM Validation Report/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FA2BA04-7187-4D7C-8104-A889816A2FDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{0FA2BA04-7187-4D7C-8104-A889816A2FDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C399B923-C87F-4410-880F-DB608C16D042}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="22320" windowHeight="13176" firstSheet="2" activeTab="5" xr2:uid="{C905B5A6-9A21-4C0A-954C-F6F13E9F5544}"/>
+    <workbookView minimized="1" xWindow="1392" yWindow="4596" windowWidth="17280" windowHeight="9060" firstSheet="2" activeTab="5" xr2:uid="{C905B5A6-9A21-4C0A-954C-F6F13E9F5544}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -7618,6 +7618,11 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55CAA6A6-CF86-41FB-8BD9-00612CE7B1AC}">
   <dimension ref="A1:D1"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.77734375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">

</xml_diff>